<commit_message>
modified:   ai-first-delivery-mumbai-gaurav/MD files/virtual-gaurav assistant.md
</commit_message>
<xml_diff>
--- a/Batch 5 Scoring.xlsx
+++ b/Batch 5 Scoring.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://onlinect-my.sharepoint.com/personal/vaishali_desai_citiustech_com/Documents/Vaishali Desai/Vaishali/Gen AI/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\GauravC2\Documents\AI FD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1CEB2ACF-CA17-42CF-BEE7-D7C57A15C499}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{943B87E4-B1E5-481B-B0FC-D4E44EEC8C57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{98998884-4A9B-461E-9B72-1E874B4C1E9D}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{98998884-4A9B-461E-9B72-1E874B4C1E9D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -540,25 +540,43 @@
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
+      <c r="B2" s="3">
+        <v>3</v>
+      </c>
+      <c r="C2" s="3">
+        <v>3</v>
+      </c>
+      <c r="D2" s="3">
+        <v>3</v>
+      </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
+      <c r="B3" s="3">
+        <v>4</v>
+      </c>
+      <c r="C3" s="3">
+        <v>3</v>
+      </c>
+      <c r="D3" s="3">
+        <v>3</v>
+      </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
+      <c r="B4" s="3">
+        <v>3</v>
+      </c>
+      <c r="C4" s="3">
+        <v>3</v>
+      </c>
+      <c r="D4" s="3">
+        <v>3</v>
+      </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
@@ -588,49 +606,85 @@
       <c r="A8" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="3"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
+      <c r="B8" s="3">
+        <v>3</v>
+      </c>
+      <c r="C8" s="3">
+        <v>3</v>
+      </c>
+      <c r="D8" s="3">
+        <v>2</v>
+      </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
+      <c r="B9" s="3">
+        <v>3</v>
+      </c>
+      <c r="C9" s="3">
+        <v>3</v>
+      </c>
+      <c r="D9" s="3">
+        <v>3</v>
+      </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="3"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
+      <c r="B10" s="3">
+        <v>4</v>
+      </c>
+      <c r="C10" s="3">
+        <v>4</v>
+      </c>
+      <c r="D10" s="3">
+        <v>3</v>
+      </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
+      <c r="B11" s="3">
+        <v>3</v>
+      </c>
+      <c r="C11" s="3">
+        <v>2</v>
+      </c>
+      <c r="D11" s="3">
+        <v>3</v>
+      </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B12" s="3"/>
-      <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
+      <c r="B12" s="3">
+        <v>3</v>
+      </c>
+      <c r="C12" s="3">
+        <v>3</v>
+      </c>
+      <c r="D12" s="3">
+        <v>3</v>
+      </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
+      <c r="B13" s="3">
+        <v>3</v>
+      </c>
+      <c r="C13" s="3">
+        <v>3</v>
+      </c>
+      <c r="D13" s="3">
+        <v>3</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>